<commit_message>
Repair Germany DSI records and site exports
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -840,29 +840,29 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': 0}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': 0}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': 0}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -1.857, 'latest_30d': -1.667, 'change_7d': 0.286, 'change_30d': 0.2, 'current_year': 2026, 'current_year_mean': -1.522}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.429, 'latest_30d': -0.067, 'change_7d': 0.429, 'change_30d': -0.8, 'current_year': 2026, 'current_year_mean': 0.411}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.571, 'latest_30d': 0.7, 'change_7d': -1, 'change_30d': 0.633, 'current_year': 2026, 'current_year_mean': 0.367}}</t>
         </is>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>-1.857</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>-1.667</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>0.286</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="X4" t="n">
         <v>2026</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>-1.522</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Refresh CA/RU/MX site data and trim early FR coverage
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -737,7 +737,7 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.714, 'latest_30d': -1.8, 'change_7d': 0, 'change_30d': -0.4, 'current_year': 2026, 'current_year_mean': -1.484}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.143, 'latest_30d': -0.333, 'change_7d': 0, 'change_30d': -0.533, 'current_year': 2026, 'current_year_mean': 0.194}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.714, 'latest_30d': 0.233, 'change_7d': 0.714, 'change_30d': -0.833, 'current_year': 2026, 'current_year_mean': 0.753}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.714, 'latest_30d': -1.833, 'change_7d': 0, 'change_30d': -0.433, 'current_year': 2026, 'current_year_mean': -1.495}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -0.433, 'change_7d': -0.143, 'change_30d': -0.467, 'current_year': 2026, 'current_year_mean': 0.097}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.143, 'latest_30d': -0.067, 'change_7d': 0.429, 'change_30d': -0.867, 'current_year': 2026, 'current_year_mean': 0.462}}</t>
         </is>
       </c>
       <c r="S3" t="n">
@@ -747,19 +747,19 @@
         <v>-1.714</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.8</v>
+        <v>-1.833</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>-0.4</v>
+        <v>-0.433</v>
       </c>
       <c r="X3" t="n">
         <v>2026</v>
       </c>
       <c r="Y3" t="n">
-        <v>-1.484</v>
+        <v>-1.495</v>
       </c>
     </row>
     <row r="4">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2012-05-24</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1211,10 +1211,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1250</v>
+        <v>848</v>
       </c>
       <c r="I8" t="n">
-        <v>5069</v>
+        <v>1560</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Secretary of State Sarai concludes visit to Ukraine and Poland</t>
+          <t>Minister Sidhu to represent Canada and advance trade efforts in People’s Republic of China</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/global-affairs/news/2026/04/secretary-of-state-sarai-concludes-visit-to-ukraine-and-poland.html</t>
+          <t>https://www.canada.ca/en/global-affairs/news/2026/04/minister-sidhu-to-represent-canada-and-advance-trade-efforts-in-peoples-republic-of-china.html</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Foreign Minister Sergey Lavrov’s opening remarks during talks with Minister of Foreign Affairs and International Cooperation of the Republic of Malawi George Tapatula Chaponda on the sidelines of the Second Ministerial Conference of the Russia-Africa Partnership Forum, Cairo, December 19, 2025</t>
+          <t>Excerpt from Foreign Minister Sergey Lavrov’ interview for Russian Public Television, Moscow, April 11, 2026</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://mid.ru/en/foreign_policy/news/2067325</t>
+          <t>https://mid.ru/en/foreign_policy/news/2093861</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>México y Nueva Zelandia celebran primer Diálogo de Alto Nivel sobre Asuntos Multilaterales</t>
+          <t>México y EE.UU. fortalecen modernización y reforzamiento de seguridad fronteriza: Grupo Binacional sobre Puentes y Cruces Internacionales</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/sre/prensa/mexico-y-nueva-zelandia-celebran-primer-dialogo-de-alto-nivel-sobre-asuntos-multilaterales?idiom=en</t>
+          <t>https://www.gob.mx/sre/prensa/mexico-y-ee-uu-fortalecen-modernizacion-y-reforzamiento-de-seguridad-fronteriza-grupo-binacional-sobre-puentes-y-cruces-internacionales?idiom=en</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild site datasets with refreshed CA/FR/RU/MX outputs
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -1408,19 +1408,19 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1180</v>
+        <v>2769</v>
       </c>
       <c r="I10" t="n">
-        <v>5207</v>
+        <v>5214</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1458,29 +1458,29 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -0.286, 'latest_30d': -0.067, 'change_7d': -0.286, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': -0.022}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.571, 'latest_30d': 0.133, 'change_7d': 0.571, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 0.043}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 3, 'latest_filled': 3, 'latest_7d': -1, 'latest_30d': -1.767, 'change_7d': 1, 'change_30d': 0.233, 'current_year': 2026, 'current_year_mean': -1.925}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1.067, 'change_7d': 1.143, 'change_30d': -0.533, 'current_year': 2026, 'current_year_mean': -0.86}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.286, 'latest_30d': 0.5, 'change_7d': -0.429, 'change_30d': 0.1, 'current_year': 2026, 'current_year_mean': 0.66}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.267, 'change_7d': -0.571, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': 0.63}}</t>
         </is>
       </c>
       <c r="S10" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.286</v>
+        <v>-0.429</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.067</v>
+        <v>-1.067</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.286</v>
+        <v>1.143</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.067</v>
+        <v>-0.533</v>
       </c>
       <c r="X10" t="n">
         <v>2026</v>
       </c>
       <c r="Y10" t="n">
-        <v>-0.022</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="11">
@@ -1614,19 +1614,19 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>489</v>
+        <v>670</v>
       </c>
       <c r="I12" t="n">
-        <v>5766</v>
+        <v>5879</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1664,29 +1664,29 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -2.286, 'latest_30d': -2.067, 'change_7d': 0.714, 'change_30d': -1.333, 'current_year': 2025, 'current_year_mean': -2.17}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.286, 'latest_30d': -1.333, 'change_7d': 0.714, 'change_30d': 0.367, 'current_year': 2025, 'current_year_mean': -1.255}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.714, 'latest_30d': -1.467, 'change_7d': 1.286, 'change_30d': -1.767, 'current_year': 2025, 'current_year_mean': -0.564}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -2.286, 'latest_30d': -2.433, 'change_7d': 0.143, 'change_30d': -0.233, 'current_year': 2026, 'current_year_mean': -2.168}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': -0.571, 'latest_30d': -0.433, 'change_7d': -0.429, 'change_30d': 0.167, 'current_year': 2026, 'current_year_mean': -0.564}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 3, 'latest_filled': 3, 'latest_7d': -0.714, 'latest_30d': -0.767, 'change_7d': -0.143, 'change_30d': -0.2, 'current_year': 2026, 'current_year_mean': -0.812}}</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
         <v>-2.286</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.067</v>
+        <v>-2.433</v>
       </c>
       <c r="V12" t="n">
-        <v>0.714</v>
+        <v>0.143</v>
       </c>
       <c r="W12" t="n">
-        <v>-1.333</v>
+        <v>-0.233</v>
       </c>
       <c r="X12" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="Y12" t="n">
-        <v>-2.17</v>
+        <v>-2.168</v>
       </c>
     </row>
     <row r="13">
@@ -1820,19 +1820,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1897</v>
+        <v>2406</v>
       </c>
       <c r="I14" t="n">
-        <v>3798</v>
+        <v>3813</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1870,29 +1870,29 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': -0.143, 'latest_30d': -0.3, 'change_7d': 0.143, 'change_30d': -0.3, 'current_year': 2026, 'current_year_mean': -0.07}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0.867, 'change_7d': -0.857, 'change_30d': 0.167, 'current_year': 2026, 'current_year_mean': 0.698}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.857, 'latest_30d': 1.433, 'change_7d': 0.857, 'change_30d': 0.533, 'current_year': 2026, 'current_year_mean': 1.36}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.143, 'latest_30d': -0.2, 'change_7d': 0.286, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': -0.069}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.286, 'latest_30d': 0.267, 'change_7d': 0.286, 'change_30d': -0.733, 'current_year': 2026, 'current_year_mean': 0.614}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 1.429, 'latest_30d': 0.733, 'change_7d': 1.857, 'change_30d': -0.7, 'current_year': 2026, 'current_year_mean': 1.168}}</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.143</v>
+        <v>0.143</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="V14" t="n">
-        <v>0.143</v>
+        <v>0.286</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.3</v>
+        <v>-0.067</v>
       </c>
       <c r="X14" t="n">
         <v>2026</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06900000000000001</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Refresh 15-country site data
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,127 +418,127 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label_zh</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>color</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>latest_date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>latest_publication_date</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>publication_days</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>calendar_days</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>latest_title</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>latest_url</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>file_json</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>file_csv</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>file_xlsx</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>is_placeholder</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>placeholder_note</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>indicators</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>latest_raw</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>latest_7d</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>latest_30d</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>change_7d</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>change_30d</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>current_year</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>current_year_mean</t>
         </is>
@@ -1211,7 +1199,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>848</v>
+        <v>912</v>
       </c>
       <c r="I8" t="n">
         <v>1560</v>
@@ -1252,29 +1240,29 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': -1, 'latest_30d': -1.6, 'change_7d': 0.571, 'change_30d': -0.967, 'current_year': 2026, 'current_year_mean': -1.141}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 3, 'latest_filled': 3, 'latest_7d': 0.429, 'latest_30d': 0.4, 'change_7d': 0.143, 'change_30d': 0.3, 'current_year': 2026, 'current_year_mean': 0.141}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': -0.286, 'latest_30d': -0.6, 'change_7d': 0.714, 'change_30d': -1.433, 'current_year': 2026, 'current_year_mean': 0.202}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.143, 'latest_30d': -0.933, 'change_7d': 1.143, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.848}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 3, 'latest_filled': 3, 'latest_7d': 0.429, 'latest_30d': 0.533, 'change_7d': 0, 'change_30d': 0.433, 'current_year': 2026, 'current_year_mean': 0.212}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': -0.286, 'latest_30d': -0.233, 'change_7d': 0, 'change_30d': -0.767, 'current_year': 2026, 'current_year_mean': 0.333}}</t>
         </is>
       </c>
       <c r="S8" t="n">
         <v>1</v>
       </c>
       <c r="T8" t="n">
-        <v>-1</v>
+        <v>0.143</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.6</v>
+        <v>-0.9330000000000001</v>
       </c>
       <c r="V8" t="n">
-        <v>0.571</v>
+        <v>1.143</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.967</v>
+        <v>-0.133</v>
       </c>
       <c r="X8" t="n">
         <v>2026</v>
       </c>
       <c r="Y8" t="n">
-        <v>-1.141</v>
+        <v>-0.848</v>
       </c>
     </row>
     <row r="9">
@@ -1321,12 +1309,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Ricorso dell’Italia contro il brevetto europeo</t>
+          <t>Accordo sul riconoscimento reciproco in materia di conversione delle patenti di guida tra l’Italia e l’Ecuador</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>http://www.esteri.it:80/MAE/IT/Sala_Stampa/ArchivioNotizie/Comunicati/2011/05/20110531_RicorsoItalia.htm</t>
+          <t>http://www.esteri.it/MAE/IT/Sala_Stampa/ArchivioNotizie/Comunicati/2011/05/20110601_patentiecuador.htm</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1417,7 +1405,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2881</v>
+        <v>3057</v>
       </c>
       <c r="I10" t="n">
         <v>5214</v>
@@ -2116,12 +2104,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Repair Canada DSI site data
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -1396,28 +1396,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2666</v>
+        <v>3057</v>
       </c>
       <c r="I10" t="n">
-        <v>5221</v>
+        <v>5214</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>G7 Rapid Response Mechanism (RRM) releases report on joint monitoring of 2025 Moldovan parliamentary elections</t>
+          <t>Minister Sidhu to represent Canada and advance trade efforts in People’s Republic of China</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/global-affairs/news/2026/04/g7-rapid-response-mechanism-rrm-releases-report-on-joint-monitoring-of-2025-moldovan-parliamentary-elections.html</t>
+          <t>https://www.canada.ca/en/global-affairs/news/2026/04/minister-sidhu-to-represent-canada-and-advance-trade-efforts-in-peoples-republic-of-china.html</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1446,29 +1446,29 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': -0.9, 'change_7d': 0.429, 'change_30d': -0.667, 'current_year': 2026, 'current_year_mean': -0.804}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 1.714, 'latest_30d': 0.833, 'change_7d': 1.429, 'change_30d': 0.367, 'current_year': 2026, 'current_year_mean': 0.729}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -0.286, 'latest_30d': 0.2, 'change_7d': -0.571, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': 0.57}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1.067, 'change_7d': 1.143, 'change_30d': -0.533, 'current_year': 2026, 'current_year_mean': -0.86}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.286, 'latest_30d': 0.5, 'change_7d': -0.429, 'change_30d': 0.1, 'current_year': 2026, 'current_year_mean': 0.66}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.267, 'change_7d': -0.571, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': 0.63}}</t>
         </is>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>-0.429</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.9</v>
+        <v>-1.067</v>
       </c>
       <c r="V10" t="n">
-        <v>0.429</v>
+        <v>1.143</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.667</v>
+        <v>-0.533</v>
       </c>
       <c r="X10" t="n">
         <v>2026</v>
       </c>
       <c r="Y10" t="n">
-        <v>-0.804</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Show France DSI from 2012 start
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -1185,7 +1185,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2022-01-01</t>
+          <t>2012-05-24</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1199,10 +1199,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>918</v>
+        <v>1320</v>
       </c>
       <c r="I8" t="n">
-        <v>1569</v>
+        <v>5078</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh CN US KR DSI data
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,127 +430,127 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label_zh</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>color</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>latest_date</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>latest_publication_date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>publication_days</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>calendar_days</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>latest_title</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>latest_url</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>file_json</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>file_csv</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>file_xlsx</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>is_placeholder</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>placeholder_note</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>indicators</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>latest_raw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>latest_7d</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>latest_30d</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>change_7d</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>change_30d</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>current_year</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>current_year_mean</t>
         </is>
@@ -572,28 +584,28 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5437</v>
+        <v>5512</v>
       </c>
       <c r="I2" t="n">
-        <v>5952</v>
+        <v>6026</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Zimbabwe National Day</t>
+          <t>Somalia National Day</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.state.gov/releases/office-of-the-spokesperson/2026/04/zimbabwe-national-day</t>
+          <t>https://www.state.gov/releases/office-of-the-spokesperson/2026/07/somalia-national-day-2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -622,29 +634,29 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.857, 'latest_30d': -0.9, 'change_7d': -0.571, 'change_30d': 0.4, 'current_year': 2026, 'current_year_mean': -0.898}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.143, 'latest_30d': 0.233, 'change_7d': -1.571, 'change_30d': 0.7, 'current_year': 2026, 'current_year_mean': -0.13}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -0.143, 'latest_30d': 0.133, 'change_7d': -0.857, 'change_30d': 0.533, 'current_year': 2026, 'current_year_mean': -0.102}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': -0.286, 'latest_30d': -0.967, 'change_7d': 0.857, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': -0.956}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.286, 'latest_30d': -0.933, 'change_7d': 0.571, 'change_30d': -0.1, 'current_year': 2026, 'current_year_mean': -0.566}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.571, 'latest_30d': -0.167, 'change_7d': 1.143, 'change_30d': 0.2, 'current_year': 2026, 'current_year_mean': -0.236}}</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.857</v>
+        <v>-0.286</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.9</v>
+        <v>-0.967</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.571</v>
+        <v>0.857</v>
       </c>
       <c r="W2" t="n">
-        <v>0.4</v>
+        <v>-0.067</v>
       </c>
       <c r="X2" t="n">
         <v>2026</v>
       </c>
       <c r="Y2" t="n">
-        <v>-0.898</v>
+        <v>-0.956</v>
       </c>
     </row>
     <row r="3">
@@ -675,28 +687,28 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3668</v>
+        <v>3739</v>
       </c>
       <c r="I3" t="n">
-        <v>8361</v>
+        <v>8466</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026年4月17日外交部发言人郭嘉昆主持例行记者会</t>
+          <t>Foreign Ministry Spokesperson Mao Ning’s Regular Press Conference on July 31, 2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.mfa.gov.cn/fyrbt_673021/jzhsl_673025/202604/t20260417_11894119.shtml</t>
+          <t>https://www.mfa.gov.cn/eng/xw/fyrbt/lxjzh/202607/t20260731_11996482.html</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -725,17 +737,17 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -1.143, 'latest_30d': -1.567, 'change_7d': 0.429, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': -1.477}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.429, 'latest_30d': -0.667, 'change_7d': -0.857, 'change_30d': -0.4, 'current_year': 2026, 'current_year_mean': -0.047}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': 0.571, 'latest_30d': 0.4, 'change_7d': -0.571, 'change_30d': -0.033, 'current_year': 2026, 'current_year_mean': 0.514}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.857, 'latest_30d': -1.6, 'change_7d': 0.429, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': -1.792}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0, 'latest_30d': 0.433, 'change_7d': -1.143, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': 0.269}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.857, 'latest_30d': 1.8, 'change_7d': 0, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 1.104}}</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T3" t="n">
-        <v>-1.143</v>
+        <v>-1.857</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.567</v>
+        <v>-1.6</v>
       </c>
       <c r="V3" t="n">
         <v>0.429</v>
@@ -747,7 +759,7 @@
         <v>2026</v>
       </c>
       <c r="Y3" t="n">
-        <v>-1.477</v>
+        <v>-1.792</v>
       </c>
     </row>
     <row r="4">
@@ -1705,28 +1717,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>5346</v>
+        <v>5479</v>
       </c>
       <c r="I13" t="n">
-        <v>9239</v>
+        <v>9345</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Foreign Minister Holds Meeting with Korea Chemical Industry Association as well as Petrochemical and Oil Refining Companies (Apr. 17)</t>
+          <t>MOFA Spokesperson’s Commentary on “Defense of Japan 2026”</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.mofa.go.kr/eng/brd/m_5676/view.do?seq=11164&amp;page=1</t>
+          <t>https://www.mofa.go.kr/eng/brd/m_5676/view.do?seq=323334&amp;page=1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1755,29 +1767,29 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1, 'change_7d': 0.429, 'change_30d': -0.267, 'current_year': 2026, 'current_year_mean': -0.527}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -0.2, 'change_7d': 0.143, 'change_30d': -0.7, 'current_year': 2026, 'current_year_mean': 0.255}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.286, 'latest_30d': -0.733, 'change_7d': 0, 'change_30d': -1.7, 'current_year': 2026, 'current_year_mean': 0.6}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -0.429, 'latest_30d': -0.133, 'change_7d': -0.429, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.324}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.857, 'latest_30d': 0.533, 'change_7d': -0.286, 'change_30d': -0.4, 'current_year': 2026, 'current_year_mean': 0.472}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 1.714, 'latest_30d': 2, 'change_7d': -0.571, 'change_30d': 0.633, 'current_year': 2026, 'current_year_mean': 1.079}}</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="T13" t="n">
         <v>-0.429</v>
       </c>
       <c r="U13" t="n">
-        <v>-1</v>
+        <v>-0.133</v>
       </c>
       <c r="V13" t="n">
-        <v>0.429</v>
+        <v>-0.429</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.267</v>
+        <v>-0.133</v>
       </c>
       <c r="X13" t="n">
         <v>2026</v>
       </c>
       <c r="Y13" t="n">
-        <v>-0.527</v>
+        <v>-0.324</v>
       </c>
     </row>
     <row r="14">
@@ -2104,12 +2116,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Refresh remaining 12 DSI country series
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -790,28 +790,28 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>4615</v>
+        <v>4863</v>
       </c>
       <c r="I4" t="n">
-        <v>7402</v>
+        <v>7508</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Statement by Foreign Minister Johann Wadephul on the ceasefire announced between Israel and Lebanon</t>
+          <t>Foreign Minister Wadephul on the situation in Ceuta</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.auswaertiges-amt.de/en/newsroom/news/ceasefire-israel-lebanon-2768008</t>
+          <t>https://www.auswaertiges-amt.de/en/newsroom/news/2780858-2780858</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -840,29 +840,29 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.714, 'latest_30d': -2.233, 'change_7d': 1.286, 'change_30d': -0.3, 'current_year': 2026, 'current_year_mean': -1.66}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.571, 'latest_30d': 0.233, 'change_7d': 0.571, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 0.387}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.857, 'latest_30d': 1.533, 'change_7d': -0.143, 'change_30d': 1.6, 'current_year': 2026, 'current_year_mean': 0.604}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': 1.286, 'latest_30d': 0.367, 'change_7d': 0.143, 'change_30d': 0.267, 'current_year': 2026, 'current_year_mean': -0.731}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.143, 'latest_30d': 0.6, 'change_7d': -2.571, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 0.443}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 1.143, 'latest_30d': 1.1, 'change_7d': 0.286, 'change_30d': -0.4, 'current_year': 2026, 'current_year_mean': 1.019}}</t>
         </is>
       </c>
       <c r="S4" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.714</v>
+        <v>1.286</v>
       </c>
       <c r="U4" t="n">
-        <v>-2.233</v>
+        <v>0.367</v>
       </c>
       <c r="V4" t="n">
-        <v>1.286</v>
+        <v>0.143</v>
       </c>
       <c r="W4" t="n">
-        <v>-0.3</v>
+        <v>0.267</v>
       </c>
       <c r="X4" t="n">
         <v>2026</v>
       </c>
       <c r="Y4" t="n">
-        <v>-1.66</v>
+        <v>-0.731</v>
       </c>
     </row>
     <row r="5">
@@ -893,28 +893,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3680</v>
+        <v>3770</v>
       </c>
       <c r="I5" t="n">
-        <v>4799</v>
+        <v>4907</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>UK Foreign Secretary to Visit Japan and Hold the Tenth Japan-UK Foreign Ministers' Strategic Dialogue</t>
+          <t>State Minister KUNIMITSU’s Attendance at the Hiroshima Peace Memorial Ceremony</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.mofa.go.jp/press/release/pressite_000001_02274.html</t>
+          <t>https://www.mofa.go.jp/press/release/pressite_000001_02569.html</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -943,29 +943,29 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': -0.429, 'latest_30d': -0.967, 'change_7d': 1, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': -0.782}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.143, 'latest_30d': -0.233, 'change_7d': 0.571, 'change_30d': -0.167, 'current_year': 2026, 'current_year_mean': -0.1}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 1.143, 'latest_30d': 0.467, 'change_7d': 1.286, 'change_30d': -0.1, 'current_year': 2026, 'current_year_mean': 0.464}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.286, 'latest_30d': -0.433, 'change_7d': 0, 'change_30d': -0.433, 'current_year': 2026, 'current_year_mean': -0.509}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.571, 'latest_30d': 0.333, 'change_7d': 0.571, 'change_30d': 0.167, 'current_year': 2026, 'current_year_mean': 0.083}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.857, 'latest_30d': 0.967, 'change_7d': -0.286, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 0.633}}</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.429</v>
+        <v>-0.286</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.967</v>
+        <v>-0.433</v>
       </c>
       <c r="V5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>0.067</v>
+        <v>-0.433</v>
       </c>
       <c r="X5" t="n">
         <v>2026</v>
       </c>
       <c r="Y5" t="n">
-        <v>-0.782</v>
+        <v>-0.509</v>
       </c>
     </row>
     <row r="6">
@@ -996,28 +996,28 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>5843</v>
+        <v>5942</v>
       </c>
       <c r="I6" t="n">
-        <v>9606</v>
+        <v>9715</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Visit of Shri Pabitra Margherita, Union Minister of State for External Affairs to Republic of Vanuatu and Tuvalu (April 22-25, 2026)</t>
+          <t>QUESTION NO. 2173 EXPLOITATION OF INDIAN WORKERS IN GULF COUNTRIES</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.mea.gov.in/dtl/41056</t>
+          <t>https://www.mea.gov.in/rajya-sabha?dtl/41630/QUESTION_NO_2173_EXPLOITATION_OF_INDIAN_WORKERS_IN_GULF_COUNTRIES</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1046,29 +1046,29 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.143, 'latest_30d': -1.167, 'change_7d': 1.857, 'change_30d': -1.133, 'current_year': 2026, 'current_year_mean': -0.413}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.286, 'latest_30d': -0.367, 'change_7d': 2.286, 'change_30d': -1, 'current_year': 2026, 'current_year_mean': 0.22}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.286, 'latest_30d': -0.333, 'change_7d': 3.286, 'change_30d': -1.2, 'current_year': 2026, 'current_year_mean': 0.147}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.143, 'latest_30d': -0.933, 'change_7d': 0.429, 'change_30d': -0.833, 'current_year': 2026, 'current_year_mean': -0.142}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0.167, 'change_7d': 0.286, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': 0.44}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1, 'latest_30d': 0.367, 'change_7d': -1.143, 'change_30d': -0.633, 'current_year': 2026, 'current_year_mean': 0.661}}</t>
         </is>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.143</v>
+        <v>-1.143</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.167</v>
+        <v>-0.9330000000000001</v>
       </c>
       <c r="V6" t="n">
-        <v>1.857</v>
+        <v>0.429</v>
       </c>
       <c r="W6" t="n">
-        <v>-1.133</v>
+        <v>-0.833</v>
       </c>
       <c r="X6" t="n">
         <v>2026</v>
       </c>
       <c r="Y6" t="n">
-        <v>-0.413</v>
+        <v>-0.142</v>
       </c>
     </row>
     <row r="7">
@@ -1099,28 +1099,28 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4699</v>
+        <v>4773</v>
       </c>
       <c r="I7" t="n">
-        <v>5822</v>
+        <v>5931</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>FCDO statement on DPRK ballistic missile launches: 19 April</t>
+          <t>We call on the transitional government of South Sudan to cooperate fully with UNMISS: UK statement at the UN Security Council</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/news/fcdo-statement-on-dprk-ballistic-missile-launches-19-april--2</t>
+          <t>https://www.gov.uk/government/speeches/we-call-on-the-transitional-government-of-south-sudan-to-cooperate-fully-with-unmiss-uk-statement-at-the-un-security-council</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1149,29 +1149,29 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -2.286, 'latest_30d': -1.033, 'change_7d': -1.714, 'change_30d': 0.667, 'current_year': 2026, 'current_year_mean': -1.202}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.143, 'latest_30d': -0.3, 'change_7d': -0.143, 'change_30d': -0.3, 'current_year': 2026, 'current_year_mean': -0.083}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.133, 'change_7d': -0.429, 'change_30d': 0.433, 'current_year': 2026, 'current_year_mean': 0}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.714, 'latest_30d': -2.033, 'change_7d': 0.286, 'change_30d': 0.567, 'current_year': 2026, 'current_year_mean': -1.743}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0.286, 'change_30d': 0.033, 'current_year': 2026, 'current_year_mean': -0.087}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1, 'latest_30d': -0.933, 'change_7d': 0.286, 'change_30d': -0.9, 'current_year': 2026, 'current_year_mean': -0.216}}</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T7" t="n">
-        <v>-2.286</v>
+        <v>-1.714</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.033</v>
+        <v>-2.033</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.714</v>
+        <v>0.286</v>
       </c>
       <c r="W7" t="n">
-        <v>0.667</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="X7" t="n">
         <v>2026</v>
       </c>
       <c r="Y7" t="n">
-        <v>-1.202</v>
+        <v>-1.743</v>
       </c>
     </row>
     <row r="8">
@@ -1202,28 +1202,28 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1320</v>
+        <v>1412</v>
       </c>
       <c r="I8" t="n">
-        <v>5078</v>
+        <v>5186</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Décès d'un soldat français dans une attaque contre la FINUL</t>
+          <t>Liban – Sixième anniversaire de l’explosion du port de Beyrouth</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.diplomatie.gouv.fr/fr/presse-et-ressources/decouvrir-et-informer/actualites/deces-d-un-soldat-francais-dans-une-attaque-contre-la-finul</t>
+          <t>https://www.diplomatie.gouv.fr/fr/presse-et-ressources/decouvrir-et-informer/actualites/liban-sixieme-anniversaire-de-l-explosion-du-port-de-beyrouth</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1252,29 +1252,29 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -2, 'latest_30d': -1.3, 'change_7d': -1.571, 'change_30d': -0.6, 'current_year': 2026, 'current_year_mean': -0.944}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.286, 'latest_30d': 0.367, 'change_7d': -0.714, 'change_30d': 0.167, 'current_year': 2026, 'current_year_mean': 0.176}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.571, 'latest_30d': 0, 'change_7d': 0, 'change_30d': -0.333, 'current_year': 2026, 'current_year_mean': 0.361}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.714, 'latest_30d': -0.167, 'change_7d': -1, 'change_30d': 0.667, 'current_year': 2026, 'current_year_mean': -0.968}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0.433, 'change_7d': -0.857, 'change_30d': 0.9, 'current_year': 2026, 'current_year_mean': -0.019}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1, 'latest_30d': 0.7, 'change_7d': -0.429, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': 0.472}}</t>
         </is>
       </c>
       <c r="S8" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>-2</v>
+        <v>-0.714</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.3</v>
+        <v>-0.167</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.571</v>
+        <v>-1</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.6</v>
+        <v>0.667</v>
       </c>
       <c r="X8" t="n">
         <v>2026</v>
       </c>
       <c r="Y8" t="n">
-        <v>-0.944</v>
+        <v>-0.968</v>
       </c>
     </row>
     <row r="9">
@@ -1305,28 +1305,28 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>3761</v>
+        <v>3866</v>
       </c>
       <c r="I9" t="n">
-        <v>5968</v>
+        <v>6075</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Ricorso dell’Italia contro il brevetto europeo</t>
+          <t>Consular visit to the minor Santoiemma in La Valletta</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>http://www.esteri.it:80/MAE/IT/Sala_Stampa/ArchivioNotizie/Comunicati/2011/05/20110531_RicorsoItalia.htm</t>
+          <t>https://www.esteri.it/en/sala_stampa/archivionotizie/comunicati/2026/08/visita-consolare-al-minore-santoiemma-a-la-valletta</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1355,29 +1355,29 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1.333, 'change_7d': 1, 'change_30d': -0.367, 'current_year': 2026, 'current_year_mean': -0.827}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.429, 'latest_30d': 0.167, 'change_7d': 2.143, 'change_30d': -0.2, 'current_year': 2026, 'current_year_mean': 0.518}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1, 'latest_30d': 0.2, 'change_7d': 0.714, 'change_30d': -0.567, 'current_year': 2026, 'current_year_mean': 0.636}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': 0.286, 'latest_30d': 0.067, 'change_7d': 0, 'change_30d': 0.4, 'current_year': 2026, 'current_year_mean': -0.401}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.4, 'change_7d': -1, 'change_30d': -0.033, 'current_year': 2026, 'current_year_mean': 0.548}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.857, 'latest_30d': 1.167, 'change_7d': -0.857, 'change_30d': 0.667, 'current_year': 2026, 'current_year_mean': 0.843}}</t>
         </is>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.429</v>
+        <v>0.286</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.333</v>
+        <v>0.067</v>
       </c>
       <c r="V9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.367</v>
+        <v>0.4</v>
       </c>
       <c r="X9" t="n">
         <v>2026</v>
       </c>
       <c r="Y9" t="n">
-        <v>-0.827</v>
+        <v>-0.401</v>
       </c>
     </row>
     <row r="10">
@@ -1408,28 +1408,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>3057</v>
+        <v>3487</v>
       </c>
       <c r="I10" t="n">
-        <v>5214</v>
+        <v>5332</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Minister Sidhu to represent Canada and advance trade efforts in People’s Republic of China</t>
+          <t>Minister LeBlanc updates Advisory Committee on Canada–U.S. Economic Relations</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/global-affairs/news/2026/04/minister-sidhu-to-represent-canada-and-advance-trade-efforts-in-peoples-republic-of-china.html</t>
+          <t>https://www.canada.ca/en/global-affairs/news/2026/08/minister-leblanc-updates-advisory-committee-on-canadaus-economic-relations.html</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1458,29 +1458,29 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1.067, 'change_7d': 1.143, 'change_30d': -0.533, 'current_year': 2026, 'current_year_mean': -0.86}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.286, 'latest_30d': 0.5, 'change_7d': -0.429, 'change_30d': 0.1, 'current_year': 2026, 'current_year_mean': 0.66}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.267, 'change_7d': -0.571, 'change_30d': 0.067, 'current_year': 2026, 'current_year_mean': 0.63}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.429, 'latest_30d': -0.2, 'change_7d': -1.857, 'change_30d': -0.1, 'current_year': 2026, 'current_year_mean': -0.509}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.571, 'latest_30d': 0.567, 'change_7d': -2.571, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': 0.716}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.571, 'latest_30d': 0.633, 'change_7d': 0, 'change_30d': 0.333, 'current_year': 2026, 'current_year_mean': 0.606}}</t>
         </is>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.429</v>
+        <v>-1.429</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.067</v>
+        <v>-0.2</v>
       </c>
       <c r="V10" t="n">
-        <v>1.143</v>
+        <v>-1.857</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.533</v>
+        <v>-0.1</v>
       </c>
       <c r="X10" t="n">
         <v>2026</v>
       </c>
       <c r="Y10" t="n">
-        <v>-0.86</v>
+        <v>-0.509</v>
       </c>
     </row>
     <row r="11">
@@ -1511,28 +1511,28 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1953</v>
+        <v>2001</v>
       </c>
       <c r="I11" t="n">
-        <v>5588</v>
+        <v>5697</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>4ª Reunião de Alto Nível do Fórum Democracia Sempre - Declaração Conjunta - Barcelona, 18 de abril de 2025</t>
+          <t>Visita do Secretário de Relações Exteriores do México, por ocasião da VI Reunião da Comissão Binacional Brasil-México — Brasília, 6 de agosto de 2026</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mre/pt-br/canais_atendimento/imprensa/notas-a-imprensa/reuniao-de-alto-nivel-democracia-sempre-declaracao-conjunta-barcelona-18-de-abril-de-2025</t>
+          <t>https://www.gov.br/mre/pt-br/canais_atendimento/imprensa/notas-a-imprensa/visita-do-secretario-de-relacoes-exteriores-do-mexico-por-ocasiao-da-vi-reuniao-da-comissao-binacional-brasil-mexico-brasilia-6-de-agosto-de-2026</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1561,29 +1561,29 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -0.867, 'change_7d': 1.429, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': -0.615}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0.143, 'latest_30d': 0.267, 'change_7d': 0.143, 'change_30d': -0.567, 'current_year': 2026, 'current_year_mean': 0.422}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.429, 'latest_30d': 0.067, 'change_7d': 0.429, 'change_30d': -0.567, 'current_year': 2026, 'current_year_mean': -0.174}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.143, 'latest_30d': -0.133, 'change_7d': 0.571, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.349}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.143, 'latest_30d': 0.567, 'change_7d': 1.286, 'change_30d': 0.433, 'current_year': 2026, 'current_year_mean': 0.427}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.714, 'latest_30d': 1.3, 'change_7d': 1.286, 'change_30d': 1.3, 'current_year': 2026, 'current_year_mean': 0.234}}</t>
         </is>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.429</v>
+        <v>0.143</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.867</v>
+        <v>-0.133</v>
       </c>
       <c r="V11" t="n">
-        <v>1.429</v>
+        <v>0.571</v>
       </c>
       <c r="W11" t="n">
-        <v>0.133</v>
+        <v>-0.133</v>
       </c>
       <c r="X11" t="n">
         <v>2026</v>
       </c>
       <c r="Y11" t="n">
-        <v>-0.615</v>
+        <v>-0.349</v>
       </c>
     </row>
     <row r="12">
@@ -1614,28 +1614,28 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>671</v>
+        <v>766</v>
       </c>
       <c r="I12" t="n">
-        <v>5883</v>
+        <v>5994</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Foreign Minister Sergey Lavrov's Remarks and Answers to Media Questions Following his Visit to the People's Republic of China, Beijing, April 15, 2026</t>
+          <t>Russian Foreign Ministry update</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://primarynewssource.org/sourcedocument/foreign-minister-sergey-lavrovs-remarks-and-answers-to-media-questions-following-his-visit-to-the-peoples-republic-of-china-beijing-april-15-2026/</t>
+          <t>https://mid.ru/ru/foreign_policy/news/2131012</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1664,29 +1664,29 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': -1, 'latest_30d': -2.267, 'change_7d': 1.571, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -2.095}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1, 'latest_30d': -0.233, 'change_7d': 1.571, 'change_30d': 0.167, 'current_year': 2026, 'current_year_mean': -0.467}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': 1, 'latest_30d': -0.533, 'change_7d': 1.857, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': -0.714}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -2.857, 'latest_30d': -1.9, 'change_7d': -0.857, 'change_30d': -0.5, 'current_year': 2026, 'current_year_mean': -1.796}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.429, 'latest_30d': -0.3, 'change_7d': -1.571, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.352}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.571, 'latest_30d': -0.4, 'change_7d': -0.286, 'change_30d': 0.033, 'current_year': 2026, 'current_year_mean': -0.505}}</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="T12" t="n">
-        <v>-1</v>
+        <v>-2.857</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.267</v>
+        <v>-1.9</v>
       </c>
       <c r="V12" t="n">
-        <v>1.571</v>
+        <v>-0.857</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.133</v>
+        <v>-0.5</v>
       </c>
       <c r="X12" t="n">
         <v>2026</v>
       </c>
       <c r="Y12" t="n">
-        <v>-2.095</v>
+        <v>-1.796</v>
       </c>
     </row>
     <row r="13">
@@ -1820,28 +1820,28 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>2411</v>
+        <v>2460</v>
       </c>
       <c r="I14" t="n">
-        <v>3820</v>
+        <v>3928</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Comunicado conjunto sobre la situación en Cuba</t>
+          <t>SRE e INAH alistan repatriación de tres piezas prehispánicas desde Estados Unidos</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/sre/prensa/comunicado-conjunto-sobre-la-situacion-en-cuba?idiom=en</t>
+          <t>https://www.gob.mx/sre/prensa/sre-e-inah-alistan-repatriacion-de-tres-piezas-prehispanicas-desde-estados-unidos?idiom=en</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1870,29 +1870,29 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.143, 'latest_30d': -0.033, 'change_7d': 0, 'change_30d': 0.2, 'current_year': 2026, 'current_year_mean': -0.056}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.857, 'latest_30d': 0.267, 'change_7d': 0.571, 'change_30d': -0.9, 'current_year': 2026, 'current_year_mean': 0.63}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': 0.571, 'latest_30d': 0.533, 'change_7d': -0.857, 'change_30d': -1, 'current_year': 2026, 'current_year_mean': 1.13}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.714, 'latest_30d': 0.267, 'change_7d': 0.714, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': 0.069}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.857, 'latest_30d': 0.733, 'change_7d': -0.286, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': 0.731}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 2, 'latest_30d': 1.4, 'change_7d': 0.143, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': 1.273}}</t>
         </is>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.143</v>
+        <v>0.714</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.033</v>
+        <v>0.267</v>
       </c>
       <c r="V14" t="n">
-        <v>0</v>
+        <v>0.714</v>
       </c>
       <c r="W14" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="X14" t="n">
         <v>2026</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.056</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -1923,28 +1923,28 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1818</v>
+        <v>1855</v>
       </c>
       <c r="I15" t="n">
-        <v>4595</v>
+        <v>4706</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Securing more fertiliser for Australian farmers</t>
+          <t>Visit to Fiji for the Pacific Islands Forum Foreign Ministers Meeting</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>http://www.foreignminister.gov.au/minister/penny-wong/media-release/securing-more-fertiliser-australian-farmers</t>
+          <t>https://www.foreignminister.gov.au/minister/penny-wong/media-release/visit-fiji-pacific-islands-forum-foreign-ministers-meeting</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1973,29 +1973,29 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.857, 'latest_30d': -1, 'change_7d': 1.429, 'change_30d': 0.633, 'current_year': 2026, 'current_year_mean': -0.71}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.857, 'latest_30d': 0.233, 'change_7d': 1.429, 'change_30d': 0.367, 'current_year': 2026, 'current_year_mean': 0.505}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 2, 'latest_30d': 1.367, 'change_7d': 0.286, 'change_30d': 1.4, 'current_year': 2026, 'current_year_mean': 0.617}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 2, 'latest_30d': 1.533, 'change_7d': 1.714, 'change_30d': 1.233, 'current_year': 2026, 'current_year_mean': -0.225}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.286, 'latest_30d': 0.933, 'change_7d': -0.857, 'change_30d': 0.3, 'current_year': 2026, 'current_year_mean': 0.674}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 2, 'latest_30d': 0.733, 'change_7d': 1, 'change_30d': -0.7, 'current_year': 2026, 'current_year_mean': 0.729}}</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.857</v>
+        <v>2</v>
       </c>
       <c r="U15" t="n">
-        <v>-1</v>
+        <v>1.533</v>
       </c>
       <c r="V15" t="n">
-        <v>1.429</v>
+        <v>1.714</v>
       </c>
       <c r="W15" t="n">
-        <v>0.633</v>
+        <v>1.233</v>
       </c>
       <c r="X15" t="n">
         <v>2026</v>
       </c>
       <c r="Y15" t="n">
-        <v>-0.71</v>
+        <v>-0.225</v>
       </c>
     </row>
     <row r="16">
@@ -2026,28 +2026,28 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1728</v>
+        <v>1755</v>
       </c>
       <c r="I16" t="n">
-        <v>5576</v>
+        <v>5680</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Comunicado conjunto sobre la situación en Cuba</t>
+          <t>His Majesty the King attends inauguration of Colombia’s new President</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>http://www.exteriores.gob.es/es/Comunicacion/Comunicados/Paginas/2026_COMUNICADOS/Comunicado-conjunto-sobre-la-situacion-en-Cuba.aspx</t>
+          <t>https://www.exteriores.gob.es/en/Comunicacion/Comunicados/Paginas/2026_COMUNICADOS/SM-el-Rey-acude-a-la-toma-de-posesion-del-nuevo-presidente-de-Colombia.aspx</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2076,29 +2076,29 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.857, 'latest_30d': -1.933, 'change_7d': 0.571, 'change_30d': 0.833, 'current_year': 2026, 'current_year_mean': -2.102}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.571, 'latest_30d': -0.267, 'change_7d': -0.286, 'change_30d': -0.2, 'current_year': 2026, 'current_year_mean': -0.074}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': 1.286, 'latest_30d': 0.3, 'change_7d': -0.286, 'change_30d': -1.133, 'current_year': 2026, 'current_year_mean': 0.741}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.429, 'latest_30d': -1.3, 'change_7d': 0.429, 'change_30d': 0.433, 'current_year': 2026, 'current_year_mean': -1.741}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': 0.028}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0, 'latest_30d': 0.433, 'change_7d': -0.857, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 0.547}}</t>
         </is>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.857</v>
+        <v>-0.429</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.933</v>
+        <v>-1.3</v>
       </c>
       <c r="V16" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="W16" t="n">
-        <v>0.833</v>
+        <v>0.433</v>
       </c>
       <c r="X16" t="n">
         <v>2026</v>
       </c>
       <c r="Y16" t="n">
-        <v>-2.102</v>
+        <v>-1.741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Include China spokesperson remarks in DSI updates
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -687,28 +687,28 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3739</v>
+        <v>3742</v>
       </c>
       <c r="I3" t="n">
-        <v>8466</v>
+        <v>8472</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Foreign Ministry Spokesperson Mao Ning’s Regular Press Conference on July 31, 2026</t>
+          <t>Foreign Ministry Spokesperson Lin Jian’s Remarks on August 6, 2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.mfa.gov.cn/eng/xw/fyrbt/lxjzh/202607/t20260731_11996482.html</t>
+          <t>https://www.mfa.gov.cn/eng/xw/fyrbt/lxjzh/202608/t20260806_11999829.html</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -737,29 +737,29 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.857, 'latest_30d': -1.6, 'change_7d': 0.429, 'change_30d': 0, 'current_year': 2026, 'current_year_mean': -1.792}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 0, 'latest_30d': 0.433, 'change_7d': -1.143, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': 0.269}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 1.857, 'latest_30d': 1.8, 'change_7d': 0, 'change_30d': 0.133, 'current_year': 2026, 'current_year_mean': 1.104}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -2.429, 'latest_30d': -2.033, 'change_7d': -0.571, 'change_30d': -0.7, 'current_year': 2026, 'current_year_mean': -1.812}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0.286, 'latest_30d': 0.733, 'change_7d': 0.714, 'change_30d': 0.6, 'current_year': 2026, 'current_year_mean': 0.266}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 1, 'latest_filled': 1, 'latest_7d': 1.571, 'latest_30d': 1.767, 'change_7d': -0.286, 'change_30d': -0.033, 'current_year': 2026, 'current_year_mean': 1.115}}</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T3" t="n">
-        <v>-1.857</v>
+        <v>-2.429</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.6</v>
+        <v>-2.033</v>
       </c>
       <c r="V3" t="n">
-        <v>0.429</v>
+        <v>-0.571</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="X3" t="n">
         <v>2026</v>
       </c>
       <c r="Y3" t="n">
-        <v>-1.792</v>
+        <v>-1.812</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Audit and complete 15-country DSI refresh
</commit_message>
<xml_diff>
--- a/data/summary.xlsx
+++ b/data/summary.xlsx
@@ -584,28 +584,28 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5512</v>
+        <v>5548</v>
       </c>
       <c r="I2" t="n">
-        <v>6026</v>
+        <v>6062</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Somalia National Day</t>
+          <t>Welcoming Talks in Caracas to Advance Venezuela’s Political Transition</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.state.gov/releases/office-of-the-spokesperson/2026/07/somalia-national-day-2</t>
+          <t>https://www.state.gov/releases/office-of-the-spokesperson/2026/08/welcoming-talks-in-caracas-to-advance-venezuelas-political-transition</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -634,29 +634,29 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': -0.286, 'latest_30d': -0.967, 'change_7d': 0.857, 'change_30d': -0.067, 'current_year': 2026, 'current_year_mean': -0.956}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.286, 'latest_30d': -0.933, 'change_7d': 0.571, 'change_30d': -0.1, 'current_year': 2026, 'current_year_mean': -0.566}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 2, 'latest_filled': 2, 'latest_7d': 0.571, 'latest_30d': -0.167, 'change_7d': 1.143, 'change_30d': 0.2, 'current_year': 2026, 'current_year_mean': -0.236}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -1.143, 'latest_30d': -1, 'change_7d': -0.143, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.968}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -0.714, 'latest_30d': -0.833, 'change_7d': 0.286, 'change_30d': -0.233, 'current_year': 2026, 'current_year_mean': -0.596}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': -1, 'latest_filled': -1, 'latest_7d': -0.571, 'latest_30d': -0.433, 'change_7d': -0.571, 'change_30d': -0.167, 'current_year': 2026, 'current_year_mean': -0.275}}</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.286</v>
+        <v>-1.143</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.967</v>
+        <v>-1</v>
       </c>
       <c r="V2" t="n">
-        <v>0.857</v>
+        <v>-0.143</v>
       </c>
       <c r="W2" t="n">
-        <v>-0.067</v>
+        <v>-0.133</v>
       </c>
       <c r="X2" t="n">
         <v>2026</v>
       </c>
       <c r="Y2" t="n">
-        <v>-0.956</v>
+        <v>-0.968</v>
       </c>
     </row>
     <row r="3">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4773</v>
+        <v>4774</v>
       </c>
       <c r="I7" t="n">
         <v>5931</v>
@@ -1149,29 +1149,29 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.714, 'latest_30d': -2.033, 'change_7d': 0.286, 'change_30d': 0.567, 'current_year': 2026, 'current_year_mean': -1.743}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0.286, 'change_30d': 0.033, 'current_year': 2026, 'current_year_mean': -0.087}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1, 'latest_30d': -0.933, 'change_7d': 0.286, 'change_30d': -0.9, 'current_year': 2026, 'current_year_mean': -0.216}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -1.286, 'latest_30d': -1.933, 'change_7d': 0.714, 'change_30d': 0.667, 'current_year': 2026, 'current_year_mean': -1.729}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': 0, 'change_7d': 0.286, 'change_30d': 0.033, 'current_year': 2026, 'current_year_mean': -0.087}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.714, 'latest_30d': -0.867, 'change_7d': 0.571, 'change_30d': -0.833, 'current_year': 2026, 'current_year_mean': -0.206}}</t>
         </is>
       </c>
       <c r="S7" t="n">
         <v>-2</v>
       </c>
       <c r="T7" t="n">
-        <v>-1.714</v>
+        <v>-1.286</v>
       </c>
       <c r="U7" t="n">
-        <v>-2.033</v>
+        <v>-1.933</v>
       </c>
       <c r="V7" t="n">
-        <v>0.286</v>
+        <v>0.714</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.667</v>
       </c>
       <c r="X7" t="n">
         <v>2026</v>
       </c>
       <c r="Y7" t="n">
-        <v>-1.743</v>
+        <v>-1.729</v>
       </c>
     </row>
     <row r="8">
@@ -1614,28 +1614,28 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="I12" t="n">
-        <v>5994</v>
+        <v>5996</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Russian Foreign Ministry update</t>
+          <t>Briefing by Deputy Director of the Information and Press Department Alexey Fadeev, Moscow, August 6, 2026</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://mid.ru/ru/foreign_policy/news/2131012</t>
+          <t>https://mid.ru/en/press_service/spokesman/briefings/2131743</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1664,29 +1664,29 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -2, 'latest_filled': -2, 'latest_7d': -2.857, 'latest_30d': -1.9, 'change_7d': -0.857, 'change_30d': -0.5, 'current_year': 2026, 'current_year_mean': -1.796}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.429, 'latest_30d': -0.3, 'change_7d': -1.571, 'change_30d': -0.133, 'current_year': 2026, 'current_year_mean': -0.352}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -0.571, 'latest_30d': -0.4, 'change_7d': -0.286, 'change_30d': 0.033, 'current_year': 2026, 'current_year_mean': -0.505}}</t>
+          <t>{'c1': {'slug': 'wdsi', 'short_label': 'WDSI', 'label': 'War-Related DSI', 'latest_raw': -3, 'latest_filled': -3, 'latest_7d': -2.714, 'latest_30d': -1.933, 'change_7d': -0.571, 'change_30d': -0.633, 'current_year': 2026, 'current_year_mean': -1.798}, 'c2': {'slug': 'edsi', 'short_label': 'EDSI', 'label': 'Economic DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': -1.143, 'latest_30d': -0.333, 'change_7d': -0.857, 'change_30d': -0.3, 'current_year': 2026, 'current_year_mean': -0.353}, 'c3': {'slug': 'odsi', 'short_label': 'ODSI', 'label': 'Other DSI', 'latest_raw': 0, 'latest_filled': 0, 'latest_7d': 0, 'latest_30d': -0.333, 'change_7d': 0.714, 'change_30d': -0.033, 'current_year': 2026, 'current_year_mean': -0.491}}</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T12" t="n">
-        <v>-2.857</v>
+        <v>-2.714</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.9</v>
+        <v>-1.933</v>
       </c>
       <c r="V12" t="n">
-        <v>-0.857</v>
+        <v>-0.571</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.5</v>
+        <v>-0.633</v>
       </c>
       <c r="X12" t="n">
         <v>2026</v>
       </c>
       <c r="Y12" t="n">
-        <v>-1.796</v>
+        <v>-1.798</v>
       </c>
     </row>
     <row r="13">

</xml_diff>